<commit_message>
fix(workbooks): revert scrub commit c4632e8; restore preScrub state
User reported both workbooks corrupted by Excel after the c4632e8 scrub
operation. openpyxl could read the post-scrub files cleanly and the
validator passed 8/0, but Excel refused to open them. Cause not fully
isolated; suspect the scrub introduced a Unicode or xlsx-schema artifact
that Excel's stricter parser rejected.

Restored both files from .preScrub-backup.xlsx:
  M67400-FO-M13020 3D MED BN-22NOV2024.xlsx
  BFR_Generator_FC2-000-05N.xlsx

This preserves all session work UP TO commit 8acdfa9 (BFRL flawless
pass + 3d MED BN FC numbers + V3 postal + Surg A=B + externalLinks
purge + H&S filter delete). Only the c4632e8 scrub commit's xlsx
edits are reverted; the audit/*.md scrub remains in place since text
files don't have Excel parser issues.

Validator: 8 PASS / 0 FAIL preserved.
</commit_message>
<xml_diff>
--- a/BFR_Generator_FC2-000-05N.xlsx
+++ b/BFR_Generator_FC2-000-05N.xlsx
@@ -1243,7 +1243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="B2:G42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="68" min="1" max="2"/>
@@ -1261,11 +1261,10 @@
     <row r="3" ht="18" customHeight="1" s="69">
       <c r="B3" s="71" t="inlineStr">
         <is>
-          <t>FC 2-000-05N · Series 100 - Operational &amp; Training Facilities · MCIPAC · Okinawa, Japan</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
+          <t>FC 2-000-05N · Series 100 — Operational &amp; Training Facilities · MCIPAC · Okinawa, Japan</t>
+        </is>
+      </c>
+    </row>
     <row r="5" ht="21.75" customHeight="1" s="69">
       <c r="B5" s="72" t="inlineStr">
         <is>
@@ -1318,7 +1317,7 @@
       </c>
       <c r="D9" s="74" t="inlineStr">
         <is>
-          <t>MCIPAC - 3d MLG / CLR-3</t>
+          <t>MCIPAC — 3d MLG / CLR-3</t>
         </is>
       </c>
       <c r="E9" s="75" t="n"/>
@@ -1348,7 +1347,7 @@
       </c>
       <c r="D11" s="74" t="inlineStr">
         <is>
-          <t>M29110 (CLB-4 - composite of M29111/12/13/14)</t>
+          <t>M29110 (CLB-4 — composite of M29111/12/13/14)</t>
         </is>
       </c>
       <c r="E11" s="75" t="n"/>
@@ -1395,7 +1394,6 @@
       <c r="F15" s="75" t="n"/>
       <c r="G15" s="75" t="n"/>
     </row>
-    <row r="16"/>
     <row r="17" ht="21.75" customHeight="1" s="69">
       <c r="B17" s="72" t="inlineStr">
         <is>
@@ -1483,23 +1481,35 @@
       <c r="D28" s="68" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="69">
-      <c r="C29" s="78" t="inlineStr"/>
+      <c r="C29" s="78" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="D29" s="79" t="inlineStr">
         <is>
-          <t>INPUT - user-editable</t>
+          <t>INPUT — user-editable</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="69">
-      <c r="C30" s="80" t="inlineStr"/>
+      <c r="C30" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="D30" s="79" t="inlineStr">
         <is>
-          <t>CALCULATED - formula</t>
+          <t>CALCULATED — formula</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="69">
-      <c r="C31" s="81" t="inlineStr"/>
+      <c r="C31" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="D31" s="79" t="inlineStr">
         <is>
           <t>OUTPUT / TOTAL</t>
@@ -1507,7 +1517,11 @@
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="69">
-      <c r="C32" s="82" t="inlineStr"/>
+      <c r="C32" s="82" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="D32" s="79" t="inlineStr">
         <is>
           <t>REVIEW REQUIRED</t>
@@ -1527,56 +1541,56 @@
     <row r="35" ht="18" customHeight="1" s="69">
       <c r="B35" s="83" t="inlineStr">
         <is>
-          <t>- FC 2-000-05N - Facility Planning for Navy and Marine Corps Shore Installations (formerly NAVFAC P-80) - Series 100, dated 11 Feb 2026</t>
+          <t>• FC 2-000-05N — Facility Planning for Navy and Marine Corps Shore Installations (formerly NAVFAC P-80) — Series 100, dated 11 Feb 2026</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1" s="69">
       <c r="B36" s="83" t="inlineStr">
         <is>
-          <t>- MCO 11000.12 - Real Property Facilities Manual, Facilities Planning and Programming</t>
+          <t>• MCO 11000.12 — Real Property Facilities Manual, Facilities Planning and Programming</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1" s="69">
       <c r="B37" s="83" t="inlineStr">
         <is>
-          <t>- MCO P11000.5x - Real Property Facilities Manual series</t>
+          <t>• MCO P11000.5x — Real Property Facilities Manual series</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1" s="69">
       <c r="B38" s="83" t="inlineStr">
         <is>
-          <t>- UFC 4-010-01 - DoD Minimum Antiterrorism Standards for Buildings</t>
+          <t>• UFC 4-010-01 — DoD Minimum Antiterrorism Standards for Buildings</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1" s="69">
       <c r="B39" s="83" t="inlineStr">
         <is>
-          <t>- UFC 4-020-01 - DoD Security Engineering Facilities Planning Manual</t>
+          <t>• UFC 4-020-01 — DoD Security Engineering Facilities Planning Manual</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1" s="69">
       <c r="B40" s="83" t="inlineStr">
         <is>
-          <t>- UFS 3-701-01 - DoD Facilities Pricing Guide (ACFs in Table 4-1)</t>
+          <t>• UFS 3-701-01 — DoD Facilities Pricing Guide (ACFs in Table 4-1)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1" s="69">
       <c r="B41" s="83" t="inlineStr">
         <is>
-          <t>- UFS 3-730-01 - Programming Cost Estimates for Military Construction</t>
+          <t>• UFS 3-730-01 — Programming Cost Estimates for Military Construction</t>
         </is>
       </c>
     </row>
     <row r="42" ht="314.9" customHeight="1" s="69">
       <c r="B42" s="83" t="inlineStr">
         <is>
-          <t>- DoD Real Property Classification System (RPCS) / iNFADS CCN module</t>
+          <t>• DoD Real Property Classification System (RPCS) / iNFADS CCN module</t>
         </is>
       </c>
     </row>
@@ -1632,7 +1646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S51"/>
+  <dimension ref="B2:S51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="68" min="1" max="1"/>
@@ -1659,11 +1673,10 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="42" customHeight="1" s="69">
       <c r="B5" s="77" t="inlineStr">
         <is>
-          <t>DATA QUALITY NOTICE - TFSMS exports are 'Published Average' snapshots and may include stale T/O lines, mis-coded FAP/collateral billets, or units detached from the parent UIC. Reconcile every row against the current Authorized Strength Report (ASR) and on-hand strength before treating these numbers as authoritative for the BFR.</t>
+          <t>DATA QUALITY NOTICE — TFSMS exports are 'Published Average' snapshots and may include stale T/O lines, mis-coded FAP/collateral billets, or units detached from the parent UIC. Reconcile every row against the current Authorized Strength Report (ASR) and on-hand strength before treating these numbers as authoritative for the BFR.</t>
         </is>
       </c>
       <c r="C5" s="75" t="n"/>
@@ -1839,7 +1852,7 @@
       <c r="R9" s="95" t="n"/>
       <c r="S9" s="91" t="inlineStr">
         <is>
-          <t>TFSMS export 25 Feb 2026; HQ Co - verify Navy RP/Chaplain billets are still chargeable to CLB-4 vs. detached.</t>
+          <t>TFSMS export 25 Feb 2026; HQ Co — verify Navy RP/Chaplain billets are still chargeable to CLB-4 vs. detached.</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1917,7 @@
       <c r="R10" s="95" t="n"/>
       <c r="S10" s="91" t="inlineStr">
         <is>
-          <t>TFSMS export 25 Feb 2026; CLC A - confirm operations chief billet (3537/0477) is filled per current ASR.</t>
+          <t>TFSMS export 25 Feb 2026; CLC A — confirm operations chief billet (3537/0477) is filled per current ASR.</t>
         </is>
       </c>
     </row>
@@ -1969,7 +1982,7 @@
       <c r="R11" s="95" t="n"/>
       <c r="S11" s="91" t="inlineStr">
         <is>
-          <t>TFSMS export 25 Feb 2026; CLC B - verify it is identical to CLC A as published; reconcile against on-hand.</t>
+          <t>TFSMS export 25 Feb 2026; CLC B — verify it is identical to CLC A as published; reconcile against on-hand.</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2047,7 @@
       <c r="R12" s="95" t="n"/>
       <c r="S12" s="91" t="inlineStr">
         <is>
-          <t>TFSMS export 25 Feb 2026; GS Co - confirm 3 collateral-duty enlisted (K15) are not double-counted in chargeable.</t>
+          <t>TFSMS export 25 Feb 2026; GS Co — confirm 3 collateral-duty enlisted (K15) are not double-counted in chargeable.</t>
         </is>
       </c>
     </row>
@@ -2609,7 +2622,6 @@
         <v/>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="B39" s="149" t="inlineStr">
         <is>
@@ -3085,7 +3097,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="B2:I41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="68" min="1" max="2"/>
@@ -3105,7 +3117,7 @@
     <row r="3" ht="18" customHeight="1" s="69">
       <c r="B3" s="71" t="inlineStr">
         <is>
-          <t>Per FC 2-000-05N §61010-3 - Personnel loading must come from an official source (ASR / TFSD).</t>
+          <t>Per FC 2-000-05N §61010-3 — Personnel loading must come from an official source (ASR / TFSD).</t>
         </is>
       </c>
     </row>
@@ -3380,8 +3392,6 @@
         <v/>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17"/>
     <row r="18" ht="21.75" customHeight="1" s="69">
       <c r="B18" s="72" t="inlineStr">
         <is>
@@ -3416,8 +3426,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22"/>
     <row r="23" ht="21.75" customHeight="1" s="69">
       <c r="B23" s="72" t="inlineStr">
         <is>
@@ -3507,8 +3515,6 @@
         <v/>
       </c>
     </row>
-    <row r="34"/>
-    <row r="35"/>
     <row r="36" ht="21.75" customHeight="1" s="69">
       <c r="B36" s="72" t="inlineStr">
         <is>
@@ -3709,7 +3715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="B2:J33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="68" min="1" max="2"/>
@@ -3724,7 +3730,7 @@
     <row r="2" ht="30" customHeight="1" s="69">
       <c r="B2" s="70" t="inlineStr">
         <is>
-          <t>BFR Calculator - Series 100</t>
+          <t>BFR Calculator — Series 100</t>
         </is>
       </c>
     </row>
@@ -3735,7 +3741,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="21.75" customHeight="1" s="69">
       <c r="B5" s="72" t="inlineStr">
         <is>
@@ -3818,7 +3823,7 @@
       <c r="I7" s="101" t="n"/>
       <c r="J7" s="106" t="inlineStr">
         <is>
-          <t>Emergency Vehicle Garage - engineering analysis required.</t>
+          <t>Emergency Vehicle Garage — engineering analysis required.</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3858,7 @@
       <c r="I8" s="101" t="n"/>
       <c r="J8" s="106" t="inlineStr">
         <is>
-          <t>Operational Vehicle Garage - sum of all type allowances + 250 SF mech room.</t>
+          <t>Operational Vehicle Garage — sum of all type allowances + 250 SF mech room.</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3927,7 @@
       <c r="I10" s="101" t="n"/>
       <c r="J10" s="106" t="inlineStr">
         <is>
-          <t>Marine Corps EOD Facility - 7,000 GSF EOD bldg + 204 GSF Haz/Flam.</t>
+          <t>Marine Corps EOD Facility — 7,000 GSF EOD bldg + 204 GSF Haz/Flam.</t>
         </is>
       </c>
     </row>
@@ -3955,7 +3960,7 @@
       <c r="I11" s="101" t="n"/>
       <c r="J11" s="106" t="inlineStr">
         <is>
-          <t>Armory - sized via Table 14345-1; engineering analysis if outside scope.</t>
+          <t>Armory — sized via Table 14345-1; engineering analysis if outside scope.</t>
         </is>
       </c>
     </row>
@@ -3987,7 +3992,7 @@
       <c r="I12" s="101" t="n"/>
       <c r="J12" s="106" t="inlineStr">
         <is>
-          <t>Marine Barracks - only if barracking is required.</t>
+          <t>Marine Barracks — only if barracking is required.</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4026,7 @@
       <c r="I13" s="101" t="n"/>
       <c r="J13" s="106" t="inlineStr">
         <is>
-          <t>Academic Instruction - # of student stations × 45 GSF.</t>
+          <t>Academic Instruction — # of student stations × 45 GSF.</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4060,7 @@
       <c r="I14" s="101" t="n"/>
       <c r="J14" s="106" t="inlineStr">
         <is>
-          <t>Applied Instruction - # of student stations × 150 GSF.</t>
+          <t>Applied Instruction — # of student stations × 150 GSF.</t>
         </is>
       </c>
     </row>
@@ -4087,7 +4092,7 @@
       <c r="I15" s="101" t="n"/>
       <c r="J15" s="106" t="inlineStr">
         <is>
-          <t>Indoor Small Arms Range - engineering analysis.</t>
+          <t>Indoor Small Arms Range — engineering analysis.</t>
         </is>
       </c>
     </row>
@@ -4119,7 +4124,7 @@
       <c r="I16" s="101" t="n"/>
       <c r="J16" s="106" t="inlineStr">
         <is>
-          <t>Range Operations Building - engineering analysis.</t>
+          <t>Range Operations Building — engineering analysis.</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4156,7 @@
       <c r="I17" s="101" t="n"/>
       <c r="J17" s="106" t="inlineStr">
         <is>
-          <t>Range Support Building - engineering analysis.</t>
+          <t>Range Support Building — engineering analysis.</t>
         </is>
       </c>
     </row>
@@ -4187,7 +4192,7 @@
       <c r="I18" s="101" t="n"/>
       <c r="J18" s="106" t="inlineStr">
         <is>
-          <t>Parade &amp; Drill Field - 1 AC per 125 personnel.</t>
+          <t>Parade &amp; Drill Field — 1 AC per 125 personnel.</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4226,7 @@
       <c r="I19" s="101" t="n"/>
       <c r="J19" s="106" t="inlineStr">
         <is>
-          <t>Confidence Course - 1 EA per complete course.</t>
+          <t>Confidence Course — 1 EA per complete course.</t>
         </is>
       </c>
     </row>
@@ -4253,98 +4258,98 @@
       <c r="I20" s="101" t="n"/>
       <c r="J20" s="106" t="inlineStr">
         <is>
-          <t>Obstacle Course - case-by-case engineering analysis.</t>
+          <t>Obstacle Course — case-by-case engineering analysis.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="68" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>214 51</t>
         </is>
       </c>
-      <c r="C21" s="68">
+      <c r="C21">
         <f>IFERROR(VLOOKUP(B21,CCN_TABLE,2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="D21" s="68">
+      <c r="D21">
         <f>IFERROR(VLOOKUP(B21,CCN_TABLE,3,FALSE),"")</f>
         <v/>
       </c>
-      <c r="E21" s="68" t="n">
+      <c r="E21" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="68" t="n">
+      <c r="G21" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="68">
+      <c r="H21">
         <f>IFERROR(E21*F21*G21,0)</f>
         <v/>
       </c>
-      <c r="J21" s="68" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>Auto Org Shop, TBD pending engineering study per FC 21451-3 (FC 200, p.188).</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="68" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>217 10</t>
         </is>
       </c>
-      <c r="C22" s="68">
+      <c r="C22">
         <f>IFERROR(VLOOKUP(B22,CCN_TABLE,2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="D22" s="68">
+      <c r="D22">
         <f>IFERROR(VLOOKUP(B22,CCN_TABLE,3,FALSE),"")</f>
         <v/>
       </c>
-      <c r="E22" s="68" t="n">
+      <c r="E22" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="68" t="n">
+      <c r="G22" t="n">
         <v>1.65</v>
       </c>
-      <c r="H22" s="68">
+      <c r="H22">
         <f>IFERROR(E22*F22*G22,0)</f>
         <v/>
       </c>
-      <c r="J22" s="68" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>Comm Maint Shop, TBD pending engineering evaluation per FC 21710-3 (FC 200, p.195).</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="68" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>441 12</t>
         </is>
       </c>
-      <c r="C23" s="68">
+      <c r="C23">
         <f>IFERROR(VLOOKUP(B23,CCN_TABLE,2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="D23" s="68">
+      <c r="D23">
         <f>IFERROR(VLOOKUP(B23,CCN_TABLE,3,FALSE),"")</f>
         <v/>
       </c>
-      <c r="E23" s="68" t="n">
+      <c r="E23" t="n">
         <v>0</v>
       </c>
-      <c r="F23" s="68" t="n">
+      <c r="F23" t="n">
         <v>0.49</v>
       </c>
-      <c r="G23" s="68" t="n">
+      <c r="G23" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="68">
+      <c r="H23">
         <f>IFERROR(E23*F23*G23,0)</f>
         <v/>
       </c>
-      <c r="J23" s="68" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>Storage AGE/MARCOR, 4-Step NSF=(CF*1.96)/SH; SH=4ft default. FC 440-2.2.1.</t>
         </is>
@@ -4356,29 +4361,29 @@
           <t>451 10</t>
         </is>
       </c>
-      <c r="C24" s="68">
+      <c r="C24">
         <f>IFERROR(VLOOKUP(B24,CCN_TABLE,2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="D24" s="68">
+      <c r="D24">
         <f>IFERROR(VLOOKUP(B24,CCN_TABLE,3,FALSE),"")</f>
         <v/>
       </c>
-      <c r="E24" s="68" t="n">
+      <c r="E24" t="n">
         <v>0</v>
       </c>
-      <c r="F24" s="68">
+      <c r="F24">
         <f>1.96/(4*9)</f>
         <v/>
       </c>
-      <c r="G24" s="68" t="n">
+      <c r="G24" t="n">
         <v>1</v>
       </c>
-      <c r="H24" s="68">
+      <c r="H24">
         <f>IFERROR(E24*F24*G24,0)</f>
         <v/>
       </c>
-      <c r="J24" s="68" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>Open Storage, NSY=(CF*1.96)/4/9. FC 45110-2.</t>
         </is>
@@ -4413,7 +4418,7 @@
         <f>IFERROR(E25*F25*G25,0)</f>
         <v/>
       </c>
-      <c r="J25" s="68" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>Dispensary TBD pending BUMED NMW HCRA per FC 500-2 (FC 500, p.1-2).</t>
         </is>
@@ -4446,7 +4451,7 @@
         <f>IFERROR(E26*F26*G26,0)</f>
         <v/>
       </c>
-      <c r="J26" s="68" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>Dental N/A for 3d Med Bn (zero dental billets). FC 500, p.9-11.</t>
         </is>
@@ -4480,7 +4485,7 @@
         <f>IFERROR(E27*F27*G27,0)</f>
         <v/>
       </c>
-      <c r="J27" s="68" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>BN/Squadron HQ 162.5 GSF/PN max per FC 61010-1.1.</t>
         </is>
@@ -4513,7 +4518,7 @@
         <f>IFERROR(E28*F28*G28,0)</f>
         <v/>
       </c>
-      <c r="J28" s="68" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>Co/Battery HQ 162.5 GSF/PN max per FC 61010-1.1.</t>
         </is>
@@ -4546,7 +4551,7 @@
         <f>IFERROR(E29*F29*G29,0)</f>
         <v/>
       </c>
-      <c r="J29" s="68" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>Garrison Aid Station Role 1, TBD per Table 61074-1. Excludes lab/radiological/surgical.</t>
         </is>
@@ -4686,7 +4691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="B2:J20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="68" min="1" max="2"/>
@@ -4712,7 +4717,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="21.75" customHeight="1" s="69">
       <c r="B5" s="72" t="inlineStr">
         <is>
@@ -5311,7 +5315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="B2:E27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="68" min="1" max="2"/>
@@ -5335,7 +5339,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="21.75" customHeight="1" s="69">
       <c r="B5" s="72" t="inlineStr">
         <is>
@@ -5387,7 +5390,7 @@
       </c>
       <c r="D8" s="117" t="inlineStr">
         <is>
-          <t>Sustainment ACF - used for SR per UFS 3-701-01 §3-3.</t>
+          <t>Sustainment ACF — used for SR per UFS 3-701-01 §3-3.</t>
         </is>
       </c>
       <c r="E8" s="96" t="n"/>
@@ -5427,7 +5430,7 @@
     <row r="11" ht="102" customHeight="1" s="69">
       <c r="B11" s="73" t="inlineStr">
         <is>
-          <t>SIOH (OCONUS - Japan)</t>
+          <t>SIOH (OCONUS — Japan)</t>
         </is>
       </c>
       <c r="C11" s="116" t="n">
@@ -5472,8 +5475,6 @@
       </c>
       <c r="E13" s="96" t="n"/>
     </row>
-    <row r="14"/>
-    <row r="15"/>
     <row r="16" ht="21.75" customHeight="1" s="69">
       <c r="B16" s="72" t="inlineStr">
         <is>
@@ -5633,7 +5634,7 @@
       </c>
       <c r="C27" s="106" t="inlineStr">
         <is>
-          <t>Sustainability - LEED Silver minimum / DoD Federal High-Performance Sustainable Buildings.</t>
+          <t>Sustainability — LEED Silver minimum / DoD Federal High-Performance Sustainable Buildings.</t>
         </is>
       </c>
       <c r="D27" s="91" t="n"/>
@@ -5682,7 +5683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J75"/>
+  <dimension ref="B2:J75"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="68" min="1" max="2"/>
@@ -5697,7 +5698,7 @@
     <row r="2" ht="30" customHeight="1" s="69">
       <c r="B2" s="70" t="inlineStr">
         <is>
-          <t>BFR Summary - Print-Ready</t>
+          <t>BFR Summary — Print-Ready</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5709,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="21.75" customHeight="1" s="69">
       <c r="B5" s="72" t="inlineStr">
         <is>
@@ -5879,7 +5879,6 @@
       <c r="H15" s="75" t="n"/>
       <c r="I15" s="75" t="n"/>
     </row>
-    <row r="16"/>
     <row r="17" ht="21.75" customHeight="1" s="69">
       <c r="B17" s="72" t="inlineStr">
         <is>
@@ -5959,8 +5958,6 @@
       <c r="H20" s="75" t="n"/>
       <c r="I20" s="96" t="n"/>
     </row>
-    <row r="21"/>
-    <row r="22"/>
     <row r="23" ht="21.75" customHeight="1" s="69">
       <c r="B23" s="72" t="inlineStr">
         <is>
@@ -6500,8 +6497,6 @@
         <v/>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40"/>
     <row r="41" ht="21.75" customHeight="1" s="69">
       <c r="B41" s="72" t="inlineStr">
         <is>
@@ -7120,8 +7115,6 @@
         <v/>
       </c>
     </row>
-    <row r="58"/>
-    <row r="59"/>
     <row r="60" ht="21.75" customHeight="1" s="69">
       <c r="B60" s="72" t="inlineStr">
         <is>
@@ -7163,7 +7156,6 @@
     <row r="68" ht="15" customHeight="1" s="69">
       <c r="B68" s="125" t="n"/>
     </row>
-    <row r="69"/>
     <row r="70" ht="21.75" customHeight="1" s="69">
       <c r="B70" s="72" t="inlineStr">
         <is>
@@ -7304,7 +7296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I1065"/>
+  <dimension ref="B2:I1065"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="68" min="1" max="2"/>
@@ -7328,11 +7320,10 @@
     <row r="3" ht="18" customHeight="1" s="69">
       <c r="B3" s="71" t="inlineStr">
         <is>
-          <t>FC 2-000-05N - Operational and Training Facilities (Marine Corps relevant CCNs).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
+          <t>FC 2-000-05N — Operational and Training Facilities (Marine Corps relevant CCNs).</t>
+        </is>
+      </c>
+    </row>
     <row r="5" ht="15" customHeight="1" s="69">
       <c r="C5" s="107" t="inlineStr">
         <is>
@@ -7516,7 +7507,7 @@
       <c r="H11" s="141" t="n"/>
       <c r="I11" s="140" t="inlineStr">
         <is>
-          <t>AREAS EXTENDING AT EACH END OF A RUNWAY. THE RUNWAY OVERRUN AREAS ARE REQUIRED TO REDUCE SERIOUS DAMAGE TO AN AIRCRAFT if THE AIRCRAFT RUNS OFF OF THE RUNWAY END DURING TAKEOFF OR LANDING.</t>
+          <t>AREAS EXTENDING AT EACH END OF A RUNWAY. THE RUNWAY OVERRUN AREAS ARE REQUIRED TO REDUCE SERIOUS DAMAGE TO AN AIRCRAFT IN THE EVENT THAT THE AIRCRAFT RUNS OFF OF THE RUNWAY END DURING TAKEOFF OR LANDING.</t>
         </is>
       </c>
     </row>
@@ -10242,7 +10233,7 @@
       <c r="H120" s="143" t="n"/>
       <c r="I120" s="143" t="inlineStr">
         <is>
-          <t>THE AIRCRAFT LINE OPERATIONS BUILDING IS USED TO CENTRALIZE GROUND OPERATIONS OF THE FLIGHT LINE. THE BUILDING IS used IN KEEPING OF SQUADRON DAILY FLIGHT BOOKS, AIRCRAFT STATUS BOARDS, AND BULLETIN BOARDS AND AS SUPPORT FOR LINE OPERATIONS PERSONNEL BY PROVIDING SHELTER, A WATER COOLER, AND A CHEMICAL TOILET.</t>
+          <t>THE AIRCRAFT LINE OPERATIONS BUILDING IS USED TO CENTRALIZE GROUND OPERATIONS OF THE FLIGHT LINE. THE BUILDING IS UTILIZED IN KEEPING OF SQUADRON DAILY FLIGHT BOOKS, AIRCRAFT STATUS BOARDS, AND BULLETIN BOARDS AND AS SUPPORT FOR LINE OPERATIONS PERSONNEL BY PROVIDING SHELTER, A WATER COOLER, AND A CHEMICAL TOILET.</t>
         </is>
       </c>
     </row>
@@ -10670,7 +10661,7 @@
       </c>
       <c r="I136" s="143" t="inlineStr">
         <is>
-          <t># of vehicles by Type A-G</t>
+          <t># of vehicles by Type A–G</t>
         </is>
       </c>
     </row>
@@ -11091,7 +11082,7 @@
       </c>
       <c r="G151" s="143" t="inlineStr">
         <is>
-          <t>Per Table 14346-1 (1-50: 75 GSF/PN; 201+: +30 GSF/PN).</t>
+          <t>Per Table 14346-1 (1–50: 75 GSF/PN; 201+: +30 GSF/PN).</t>
         </is>
       </c>
       <c r="H151" s="143" t="n">
@@ -13232,7 +13223,7 @@
       </c>
       <c r="D235" s="143" t="inlineStr">
         <is>
-          <t>Small Arms Range - Indoor</t>
+          <t>Small Arms Range — Indoor</t>
         </is>
       </c>
       <c r="E235" s="143" t="inlineStr">
@@ -14575,7 +14566,7 @@
       <c r="H287" s="143" t="n"/>
       <c r="I287" s="143" t="inlineStr">
         <is>
-          <t>A FIRE AND MOVEMENT RANGE IS DESIGNED FOR TRAINING INDIVIDUAL AND BUDDY/TEAM FIRE AND MOVEMENT TECHNIQUES. THE TEAM NEGOTIATES MANEUVER using COVER AND CONCEALMENT TECHNIQUES.</t>
+          <t>A FIRE AND MOVEMENT RANGE IS DESIGNED FOR TRAINING INDIVIDUAL AND BUDDY/TEAM FIRE AND MOVEMENT TECHNIQUES. THE TEAM NEGOTIATES MANEUVER UTILIZING COVER AND CONCEALMENT TECHNIQUES.</t>
         </is>
       </c>
     </row>
@@ -16029,7 +16020,7 @@
       <c r="H343" s="143" t="n"/>
       <c r="I343" s="143" t="inlineStr">
         <is>
-          <t>A BUILDING OR use IN A BUILDING USED AS AN ENGINE TEST CELL FOR EITHER IN-FRAME OR OUT- OF-FRAME ENGINE TESTING. SOMETIMES REFERRED TO AS A "HUSH HOUSE."</t>
+          <t>A BUILDING OR UTILIZATION IN A BUILDING USED AS AN ENGINE TEST CELL FOR EITHER IN-FRAME OR OUT- OF-FRAME ENGINE TESTING. SOMETIMES REFERRED TO AS A "HUSH HOUSE."</t>
         </is>
       </c>
     </row>
@@ -16429,7 +16420,7 @@
       <c r="H359" s="143" t="n"/>
       <c r="I359" s="143" t="inlineStr">
         <is>
-          <t>PROVIDES SPACE ASSOCIATED WITH PROCESSING JET, TURBOJET, AND RECIPROCATING TYPE AVIATION ENGINES in OVERHAUL, LOW TIME REPAIR, COMPLETE REPAIR, AND MAJOR INSPECTION. THE WORK FUNCTIONS PERFORMED WITHIN THIS SPACE INCLUDE UNCANNING, DISASSEMBLY, CLEANING, MATERIAL EXAMINATION, PARTS RECONDITIONING, SUBASSEMBLY, FINAL ASSEMBLY AND PRESERVATION.</t>
+          <t>PROVIDES SPACE ASSOCIATED WITH PROCESSING JET, TURBOJET, AND RECIPROCATING TYPE AVIATION ENGINES IN TERMS OF OVERHAUL, LOW TIME REPAIR, COMPLETE REPAIR, AND MAJOR INSPECTION. THE WORK FUNCTIONS PERFORMED WITHIN THIS SPACE INCLUDE UNCANNING, DISASSEMBLY, CLEANING, MATERIAL EXAMINATION, PARTS RECONDITIONING, SUBASSEMBLY, FINAL ASSEMBLY AND PRESERVATION.</t>
         </is>
       </c>
     </row>
@@ -18179,7 +18170,7 @@
       <c r="H429" s="143" t="n"/>
       <c r="I429" s="143" t="inlineStr">
         <is>
-          <t>THE FUNCTION OF A MARINE RAILWAY IS TO BRING A VESSEL OUT OF THE WATER for MAKING ALL PARTS AVAILABLE FOR OVERHAUL, AND TO RETURN THE VESSEL TO THE WATER WHEN THE WORK IS FINISHED.</t>
+          <t>THE FUNCTION OF A MARINE RAILWAY IS TO BRING A VESSEL OUT OF THE WATER FOR THE PURPOSE OF MAKING ALL PARTS AVAILABLE FOR OVERHAUL, AND TO RETURN THE VESSEL TO THE WATER WHEN THE WORK IS FINISHED.</t>
         </is>
       </c>
     </row>
@@ -18929,7 +18920,7 @@
       <c r="H459" s="143" t="n"/>
       <c r="I459" s="143" t="inlineStr">
         <is>
-          <t>THE PRIMARY FUNCTION OF THIS FACILITY IS TO WASH DOWN LANDING CRAFT AIR CUSHIONS (LCAC) VEHICLES AFTER EVERY MISSION to REMOVE SAND AND SALT SPRAY.</t>
+          <t>THE PRIMARY FUNCTION OF THIS FACILITY IS TO WASH DOWN LANDING CRAFT AIR CUSHIONS (LCAC) VEHICLES AFTER EVERY MISSION IN ORDER TO REMOVE SAND AND SALT SPRAY.</t>
         </is>
       </c>
     </row>
@@ -20045,7 +20036,7 @@
       <c r="H503" s="143" t="n"/>
       <c r="I503" s="143" t="inlineStr">
         <is>
-          <t>THIS FACILITY IS REQUIRED IN CONJUNCTION WITH CONSTRUCTION/WEIGHT-HANDLING EQUIPMENT SHOP, CATEGORY CODE 218 20 for PROTECTION OF EQUIPMENT AWAITING REPAIRS.</t>
+          <t>THIS FACILITY IS REQUIRED IN CONJUNCTION WITH CONSTRUCTION/WEIGHT-HANDLING EQUIPMENT SHOP, CATEGORY CODE 218 20 FOR THE PURPOSE OF PROTECTION OF EQUIPMENT AWAITING REPAIRS.</t>
         </is>
       </c>
     </row>
@@ -21895,7 +21886,7 @@
       <c r="H577" s="143" t="n"/>
       <c r="I577" s="143" t="inlineStr">
         <is>
-          <t>THIS FACILITY IS USED FOR RESEARCH, DEVELOPMENT, TEST AND EVALUATION OF NAVAL SYSTEMS WHICH used SEVERAL OF THE SCIENCES IN A COMBINED SYSTEM APPLIED DIRECTLY TO A FLEET PROBLEM OR AREA OF RDAT&amp;E. IT IS ALSO USED TO SUPPORT RESEARCH, DEVELOPMENT, TEST AND EVALUATION OF NAVAL SYSTEMS WHICH DO NOT LOGICALLY FIT THE OTHER CATEGORIES OF RDAT&amp;E.</t>
+          <t>THIS FACILITY IS USED FOR RESEARCH, DEVELOPMENT, TEST AND EVALUATION OF NAVAL SYSTEMS WHICH UTILIZED SEVERAL OF THE SCIENCES IN A COMBINED SYSTEM APPLIED DIRECTLY TO A FLEET PROBLEM OR AREA OF RDAT&amp;E. IT IS ALSO USED TO SUPPORT RESEARCH, DEVELOPMENT, TEST AND EVALUATION OF NAVAL SYSTEMS WHICH DO NOT LOGICALLY FIT THE OTHER CATEGORIES OF RDAT&amp;E.</t>
         </is>
       </c>
     </row>
@@ -22020,7 +22011,7 @@
       <c r="H582" s="143" t="n"/>
       <c r="I582" s="143" t="inlineStr">
         <is>
-          <t>THIS FACILITY SUPPORTS RESEARCH, DEVELOPMENT, TEST AND EVALUATION IN THE AREAS OF INFORMATION PROCESSING AND DATA HANDLING, ESPECIALLY WHEN CONCERNED WITH IDENTIFICATION OF CONDITIONS RESPONSIBLE FOR GIVEN DATA CONFIGURATIONS. MATHEMATICAL DATA ANALYSIS using BOTH DIGITAL AND ANALOG COMPUTERS TO RESEARCH, DEVELOP, TEST AND EVALUATE NEW NAVAL SYSTEMS</t>
+          <t>THIS FACILITY SUPPORTS RESEARCH, DEVELOPMENT, TEST AND EVALUATION IN THE AREAS OF INFORMATION PROCESSING AND DATA HANDLING, ESPECIALLY WHEN CONCERNED WITH IDENTIFICATION OF CONDITIONS RESPONSIBLE FOR GIVEN DATA CONFIGURATIONS. MATHEMATICAL DATA ANALYSIS UTILIZING BOTH DIGITAL AND ANALOG COMPUTERS TO RESEARCH, DEVELOP, TEST AND EVALUATE NEW NAVAL SYSTEMS</t>
         </is>
       </c>
     </row>
@@ -22045,7 +22036,7 @@
       <c r="H583" s="143" t="n"/>
       <c r="I583" s="143" t="inlineStr">
         <is>
-          <t>THIS FACILITY IS USED TO ACCOMPLISH RDT+E IN MARINE BIOSYSTEMS, ENVIRONMENTAL PROTECTION AND MANAGEMENT, DEVELOPMENT OF ANALYTICAL SYSTEMS FOR EVALUATION OF THE OCEAN ENVIRONMENT, STUDIES OF WAVE DYNAMICS, CURRENT FLOW, THERMOCLINES, CHEMICAL VARIANCES, AS WELL AS DEVELOPMENT OF NEW TECHNIQUES AND EQUIPMENT TO INCREASE MAN'S KNOWLEDGE AND use OF THE TOTAL OCEAN ENVIRONMENT.</t>
+          <t>THIS FACILITY IS USED TO ACCOMPLISH RDT+E IN MARINE BIOSYSTEMS, ENVIRONMENTAL PROTECTION AND MANAGEMENT, DEVELOPMENT OF ANALYTICAL SYSTEMS FOR EVALUATION OF THE OCEAN ENVIRONMENT, STUDIES OF WAVE DYNAMICS, CURRENT FLOW, THERMOCLINES, CHEMICAL VARIANCES, AS WELL AS DEVELOPMENT OF NEW TECHNIQUES AND EQUIPMENT TO INCREASE MAN'S KNOWLEDGE AND UTILIZATION OF THE TOTAL OCEAN ENVIRONMENT.</t>
         </is>
       </c>
     </row>
@@ -22195,7 +22186,7 @@
       <c r="H589" s="143" t="n"/>
       <c r="I589" s="143" t="inlineStr">
         <is>
-          <t>THIS FACILITY IS used IN CONDUCTING RESEARCH, DEVELOPMENT, TEST AND EVALUATION OF AERODYNAMIC DESIGN OF AIRCRAFT AND WEAPONS SYSTEMS AND NAVIGATIONAL SYSTEMS.</t>
+          <t>THIS FACILITY IS UTILIZED IN CONDUCTING RESEARCH, DEVELOPMENT, TEST AND EVALUATION OF AERODYNAMIC DESIGN OF AIRCRAFT AND WEAPONS SYSTEMS AND NAVIGATIONAL SYSTEMS.</t>
         </is>
       </c>
     </row>
@@ -22720,7 +22711,7 @@
       <c r="H610" s="143" t="n"/>
       <c r="I610" s="143" t="inlineStr">
         <is>
-          <t>THIS FACILITY IS USED TO SUPPORT RESEARCH, DEVELOPMENT, TEST AND EVALUATION OF PROPULSION SYSTEMS to DETERMINE OPERATIONAL CAPABILITIES AND IN STUDYING THE ACOUSTICS AND ELECTROMAGNETIC NOISE EFFECTS ON PERFORMANCE AND EFFICIENCY OF DRIVE UNITS.</t>
+          <t>THIS FACILITY IS USED TO SUPPORT RESEARCH, DEVELOPMENT, TEST AND EVALUATION OF PROPULSION SYSTEMS IN ORDER TO DETERMINE OPERATIONAL CAPABILITIES AND IN STUDYING THE ACOUSTICS AND ELECTROMAGNETIC NOISE EFFECTS ON PERFORMANCE AND EFFICIENCY OF DRIVE UNITS.</t>
         </is>
       </c>
     </row>
@@ -22745,7 +22736,7 @@
       <c r="H611" s="143" t="n"/>
       <c r="I611" s="143" t="inlineStr">
         <is>
-          <t>THIS FACILITY IS USED TO SUPPORT RESEARCH, DEVELOPMENT, TEST, AND EVALUATION OF PROPULSION FUELS to MAXIMIZE A PROPULSION SYSTEM'S OPERATIONAL CHARACTERISTICS. THIS FACILITY WOULD ALSO SUPPORT INVESTIGATION INTO NEW FUELS AND PROPULSIVE ENERGY SYSTEMS INCLUDING CONTROLLED NUCLEAR ENERGY.</t>
+          <t>THIS FACILITY IS USED TO SUPPORT RESEARCH, DEVELOPMENT, TEST, AND EVALUATION OF PROPULSION FUELS IN ORDER TO MAXIMIZE A PROPULSION SYSTEM'S OPERATIONAL CHARACTERISTICS. THIS FACILITY WOULD ALSO SUPPORT INVESTIGATION INTO NEW FUELS AND PROPULSIVE ENERGY SYSTEMS INCLUDING CONTROLLED NUCLEAR ENERGY.</t>
         </is>
       </c>
     </row>
@@ -24195,7 +24186,7 @@
       <c r="H669" s="143" t="n"/>
       <c r="I669" s="143" t="inlineStr">
         <is>
-          <t>A HIGH-EXPLOSIVE MAGAZINE IS USED FOR THE STORAGE OF HAZARD CLASS 1 DIVISION 1 (CH/D 1.1) ENERGETIC MATERIALS. EXAMPLES OF CH/D 1.1 MATERIALS ARE: BOMBS, MISSILES, WARHEADS, NAVAL MINES, DEMOLITION CHARGES. HC/D 1.3 AND 1.4 ENERGETICS MAY ALSO BE STORED IN A HIGH EXPLOSIVE MAGAZINE WHEN THE use REQUIRES IT AND COMPATIBILITY ALLOWS IT.</t>
+          <t>A HIGH-EXPLOSIVE MAGAZINE IS USED FOR THE STORAGE OF HAZARD CLASS 1 DIVISION 1 (CH/D 1.1) ENERGETIC MATERIALS. EXAMPLES OF CH/D 1.1 MATERIALS ARE: BOMBS, MISSILES, WARHEADS, NAVAL MINES, DEMOLITION CHARGES. HC/D 1.3 AND 1.4 ENERGETICS MAY ALSO BE STORED IN A HIGH EXPLOSIVE MAGAZINE WHEN THE UTILIZATION REQUIRES IT AND COMPATIBILITY ALLOWS IT.</t>
         </is>
       </c>
     </row>
@@ -24653,7 +24644,7 @@
       <c r="H687" s="143" t="n"/>
       <c r="I687" s="143" t="inlineStr">
         <is>
-          <t>THIS FACILITY INCLUDES GENERAL- PURPOSE WAREHOUSES DESIGNATED AS STORAGE AREAS FOR MARINE CORPS OWNED MATERIAL IN SUPPORT OF LOGISTIC SUPPORT BASE MISSION AS INTEGRATED MATERIAL MANAGERS. ALSO INCLUDED IS THE SPACE used IN SUPPORT OF PRE-POSITIONED WAR RESERVE STOCKS.</t>
+          <t>THIS FACILITY INCLUDES GENERAL- PURPOSE WAREHOUSES DESIGNATED AS STORAGE AREAS FOR MARINE CORPS OWNED MATERIAL IN SUPPORT OF LOGISTIC SUPPORT BASE MISSION AS INTEGRATED MATERIAL MANAGERS. ALSO INCLUDED IS THE SPACE UTILIZED IN SUPPORT OF PRE-POSITIONED WAR RESERVE STOCKS.</t>
         </is>
       </c>
     </row>
@@ -25502,7 +25493,7 @@
       <c r="H720" s="143" t="n"/>
       <c r="I720" s="143" t="inlineStr">
         <is>
-          <t>A STAND ALONE FACILITY SOLELY for DESTRUCTION OF CLASSIFIED MATERIALS EITHER THROUGH INCINERATION OR SHREDDING.</t>
+          <t>A STAND ALONE FACILITY SOLELY FOR THE PURPOSE OF DESTRUCTION OF CLASSIFIED MATERIALS EITHER THROUGH INCINERATION OR SHREDDING.</t>
         </is>
       </c>
     </row>
@@ -25527,7 +25518,7 @@
       <c r="H721" s="143" t="n"/>
       <c r="I721" s="143" t="inlineStr">
         <is>
-          <t>NAVAL LEGAL SERVICE OFFICES (NLSO), REGIONAL LEGAL SERVICE OFFICES (RLSO), JUDICIARY OFFICES, AND CLAIMS CENTERS PROVIDE LEGAL SERVICES TO COMMAND AND INDIVIDUAL CLIENTS. THESE SERVICES INCLUDE SAFE AND SECURE TRIALS BY COURT-MARTIAL, ADMINISTRATIVE DISCHARGE PROCEEDINGS AND OTHER PERSONNEL ACTIONS, ADJUDICATION OF CLAIMS, LEGAL ASSISTANCE, AND COMMAND ADVICE.</t>
+          <t>NAVAL LEGAL SERVICE OFFICES (NLSO), REGIONAL LEGAL SERVICE OFFICES (RLSO), JUDICIARY OFFICES, AND CLAIMS CENTERS PROVIDE COMPREHENSIVE LEGAL SERVICES TO COMMAND AND INDIVIDUAL CLIENTS. THESE SERVICES INCLUDE SAFE AND SECURE TRIALS BY COURT-MARTIAL, ADMINISTRATIVE DISCHARGE PROCEEDINGS AND OTHER PERSONNEL ACTIONS, ADJUDICATION OF CLAIMS, LEGAL ASSISTANCE, AND COMMAND ADVICE.</t>
         </is>
       </c>
     </row>
@@ -25751,7 +25742,7 @@
       <c r="H729" s="143" t="n"/>
       <c r="I729" s="143" t="inlineStr">
         <is>
-          <t>UNDERGROUND ADMINISTRATIVE FACILITY, used WHERE SECURITY PROVIDED BY UNDERGROUND LOCATION IS WARRANTED AND APPROVED BY HIGHER HEADQUARTERS.</t>
+          <t>UNDERGROUND ADMINISTRATIVE FACILITY, UTILIZED WHERE SECURITY PROVIDED BY UNDERGROUND LOCATION IS WARRANTED AND APPROVED BY HIGHER HEADQUARTERS.</t>
         </is>
       </c>
     </row>
@@ -25776,7 +25767,7 @@
       <c r="H730" s="143" t="n"/>
       <c r="I730" s="143" t="inlineStr">
         <is>
-          <t>UNDERGROUND ADMINISTRATIVE STORAGE FACILITY, used WHERE SECURITY PROVIDED BY UNDERGROUND LOCATION IS WARRANTED AND APPROVED BY HIGHER HEADQUARTERS.</t>
+          <t>UNDERGROUND ADMINISTRATIVE STORAGE FACILITY, UTILIZED WHERE SECURITY PROVIDED BY UNDERGROUND LOCATION IS WARRANTED AND APPROVED BY HIGHER HEADQUARTERS.</t>
         </is>
       </c>
     </row>
@@ -28376,7 +28367,7 @@
       <c r="H834" s="143" t="n"/>
       <c r="I834" s="143" t="inlineStr">
         <is>
-          <t>THE MWR MILITARY RECREATION CENTER (MRC) HAS INCORPORATED THE FEATURES AND FUNCTIONS OF THE FLEET RECREATION CENTER to DEFINE A FACILITY THAT SERVES THE RECREATIONAL NEEDS OF BOTH SHIP-BASED ENLISTED PERSONNEL AS WELL AS THOSE LIVING IN BACHELOR ENLISTED QUARTERS. THEY CONSIST OF SERVICES, FACILITIES, AND PROGRAMS INTENDED TO PROVIDE ALCOHOL-FREE AND TOBACCO-FREE RECREATIONAL ALTERNATIVES FOR 17- TO 25-YEAR OLDS. ALSO KNOWN AS LIBERTY OR SINGLE SAILOR CENTERS.</t>
+          <t>THE MWR MILITARY RECREATION CENTER (MRC) HAS INCORPORATED THE FEATURES AND FUNCTIONS OF THE FLEET RECREATION CENTER IN ORDER TO DEFINE A FACILITY THAT SERVES THE RECREATIONAL NEEDS OF BOTH SHIP-BASED ENLISTED PERSONNEL AS WELL AS THOSE LIVING IN BACHELOR ENLISTED QUARTERS. THEY CONSIST OF SERVICES, FACILITIES, AND PROGRAMS INTENDED TO PROVIDE ALCOHOL-FREE AND TOBACCO-FREE RECREATIONAL ALTERNATIVES FOR 17- TO 25-YEAR OLDS. ALSO KNOWN AS LIBERTY OR SINGLE SAILOR CENTERS.</t>
         </is>
       </c>
     </row>
@@ -28826,7 +28817,7 @@
       <c r="H852" s="143" t="n"/>
       <c r="I852" s="143" t="inlineStr">
         <is>
-          <t>THIS FACILITY IS INTENDED TO PROVIDE FACILITIES FOR THE ADVANCEMENT OF THE ACADEMIC, TECHNICAL, AND VOCATIONAL EDUCATION OF MILITARY PERSONNEL OF ALL GRADES AND RANKS to ENHANCE THEIR POTENTIAL TO THE SERVICE.</t>
+          <t>THIS FACILITY IS INTENDED TO PROVIDE FACILITIES FOR THE ADVANCEMENT OF THE ACADEMIC, TECHNICAL, AND VOCATIONAL EDUCATION OF MILITARY PERSONNEL OF ALL GRADES AND RANKS IN ORDER TO ENHANCE THEIR POTENTIAL TO THE SERVICE.</t>
         </is>
       </c>
     </row>
@@ -30401,7 +30392,7 @@
       <c r="H915" s="143" t="n"/>
       <c r="I915" s="143" t="inlineStr">
         <is>
-          <t>PUMP STATIONS ARE used TO PUMP CONDENSED STEAM (CONDENSATE) BACK TO THE STEAM PLANT OR OTHER FACILITY.</t>
+          <t>PUMP STATIONS ARE UTILIZED TO PUMP CONDENSED STEAM (CONDENSATE) BACK TO THE STEAM PLANT OR OTHER FACILITY.</t>
         </is>
       </c>
     </row>
@@ -32126,7 +32117,7 @@
       <c r="H984" s="143" t="n"/>
       <c r="I984" s="143" t="inlineStr">
         <is>
-          <t>A RAMP, USUALLY CONCRETE OR STEEL/IRON THAT IS used TO ASSIST IN THE LOADING OF TRUCKS AND RAILCARS.</t>
+          <t>A RAMP, USUALLY CONCRETE OR STEEL/IRON THAT IS UTILIZED TO ASSIST IN THE LOADING OF TRUCKS AND RAILCARS.</t>
         </is>
       </c>
     </row>
@@ -32676,7 +32667,7 @@
       <c r="H1006" s="143" t="n"/>
       <c r="I1006" s="143" t="inlineStr">
         <is>
-          <t>A STORM WATER RETENTION POND IS used TO CONTAIN AND CONTROL STORM WATER RUNOFF AT A PREDETERMINED RATE.</t>
+          <t>A STORM WATER RETENTION POND IS UTILIZED TO CONTAIN AND CONTROL STORM WATER RUNOFF AT A PREDETERMINED RATE.</t>
         </is>
       </c>
     </row>
@@ -33476,7 +33467,7 @@
       <c r="H1038" s="143" t="n"/>
       <c r="I1038" s="143" t="inlineStr">
         <is>
-          <t>WELLS INSTALLED AROUND A SITE to DETECT THE DISCHARGE OF ANY LEACHATE. SAMPLES FROM THE WELLS SHOULD BE ANALYZED PRIOR TO THE DISPOSAL OF ANY WASTE to ESTABLISH BASELINE DATA.</t>
+          <t>WELLS INSTALLED AROUND A SITE IN ORDER TO DETECT THE DISCHARGE OF ANY LEACHATE. SAMPLES FROM THE WELLS SHOULD BE ANALYZED PRIOR TO THE DISPOSAL OF ANY WASTE IN ORDER TO ESTABLISH BASELINE DATA.</t>
         </is>
       </c>
     </row>

</xml_diff>